<commit_message>
stalbezetting en systeemstatus toegevoegd aan leli sphere
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/luchtzuiveringssysteem/luchtzuiveringssysteem.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/luchtzuiveringssysteem/luchtzuiveringssysteem.xlsx
@@ -4353,7 +4353,7 @@
         <v>null</v>
       </c>
       <c r="M45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N45" t="str">
         <v>null</v>
@@ -4442,7 +4442,7 @@
         <v>null</v>
       </c>
       <c r="M46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N46" t="str">
         <v>null</v>
@@ -7382,7 +7382,7 @@
         <v>null</v>
       </c>
       <c r="N79" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
       </c>
       <c r="O79" t="str">
         <v>null</v>

</xml_diff>